<commit_message>
fix(gui): improve large signal workflows
</commit_message>
<xml_diff>
--- a/tests/01.data/sample_automotive_signals_2_tab_new.xlsx
+++ b/tests/01.data/sample_automotive_signals_2_tab_new.xlsx
@@ -151,16 +151,16 @@
     </row>
     <row r="6">
       <c r="A6">
-        <v>0.3</v>
+        <v>0.4</v>
       </c>
       <c r="B6">
-        <v>980</v>
+        <v>1120</v>
       </c>
       <c r="C6">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="D6">
-        <v>9</v>
+        <v>14</v>
       </c>
       <c r="E6">
         <v>1</v>
@@ -171,41 +171,21 @@
     </row>
     <row r="7">
       <c r="A7">
-        <v>0.4</v>
+        <v>0.5</v>
       </c>
       <c r="B7">
-        <v>1120</v>
+        <v>1290</v>
       </c>
       <c r="C7">
-        <v>9</v>
+        <v>14</v>
       </c>
       <c r="D7">
-        <v>14</v>
+        <v>19</v>
       </c>
       <c r="E7">
         <v>1</v>
       </c>
       <c r="F7">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8">
-        <v>0.5</v>
-      </c>
-      <c r="B8">
-        <v>1290</v>
-      </c>
-      <c r="C8">
-        <v>14</v>
-      </c>
-      <c r="D8">
-        <v>19</v>
-      </c>
-      <c r="E8">
-        <v>1</v>
-      </c>
-      <c r="F8">
         <v>1</v>
       </c>
     </row>

</xml_diff>